<commit_message>
fix: update Aciclovir.pkml in TestProject and all related references/tests
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/Applications.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/Applications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://esqlabs.sharepoint.com/sites/Services/Freigegebene Dokumente/_Project_template_V02.00/WP1_V00.01/Parameters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\update-aciclovir-pkml\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="145" documentId="13_ncr:1_{74401FE8-0DB7-4671-9034-D4AD97DAF165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE66B4D0-8183-45FE-8047-14DAA08B635C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{880F1CD1-70BF-4F87-A887-E5413A05C154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9020" yWindow="9480" windowWidth="28800" windowHeight="15290" tabRatio="965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1680" yWindow="870" windowWidth="27640" windowHeight="19270" tabRatio="965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aciclovir_iv_250mg" sheetId="14" r:id="rId1"/>
@@ -54,7 +54,7 @@
     <t>mg</t>
   </si>
   <si>
-    <t>Applications|IV 250mg 10min|Application_1|ProtocolSchemaItem</t>
+    <t>Events|IV 250mg 10min|Application_1|ProtocolSchemaItem</t>
   </si>
 </sst>
 </file>
@@ -104,9 +104,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBC36B16-DE46-4C6E-A6ED-9C66C3DB41B7}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="89.81640625" bestFit="1" customWidth="1"/>
@@ -424,24 +423,6 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C7" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C11" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -687,15 +668,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="398d2b5b-77f8-4c5f-a794-3d35ce849315">
@@ -704,6 +676,15 @@
     <TaxCatchAll xmlns="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -726,14 +707,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{253E2BCE-BEE3-46CA-82C7-E211846F5250}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D118C015-E179-46FB-B6E8-2D926D65EB7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -742,4 +715,12 @@
     <ds:schemaRef ds:uri="1c52e43a-7a2d-43c4-9ede-f251c929c0a1"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{253E2BCE-BEE3-46CA-82C7-E211846F5250}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix failing tests and Aciclovir.pkml for ospsuite v12.4.2.9011 (#999)
* fix: failing tests due to ospsuiteR v 12.4.2.9011 update

* fix: update Aciclovir.pkml in TestProject and all related references/tests

* fix: set TestScenario output path in Scenarios.xlsx

* fix: update config-json snapshot for TestScenario output

* fix: skip macos snapshot test create-plots-from-excel
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/Applications.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/Applications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://esqlabs.sharepoint.com/sites/Services/Freigegebene Dokumente/_Project_template_V02.00/WP1_V00.01/Parameters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\update-aciclovir-pkml\inst\extdata\examples\TestProject\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="145" documentId="13_ncr:1_{74401FE8-0DB7-4671-9034-D4AD97DAF165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE66B4D0-8183-45FE-8047-14DAA08B635C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{880F1CD1-70BF-4F87-A887-E5413A05C154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9020" yWindow="9480" windowWidth="28800" windowHeight="15290" tabRatio="965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1680" yWindow="870" windowWidth="27640" windowHeight="19270" tabRatio="965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aciclovir_iv_250mg" sheetId="14" r:id="rId1"/>
@@ -54,7 +54,7 @@
     <t>mg</t>
   </si>
   <si>
-    <t>Applications|IV 250mg 10min|Application_1|ProtocolSchemaItem</t>
+    <t>Events|IV 250mg 10min|Application_1|ProtocolSchemaItem</t>
   </si>
 </sst>
 </file>
@@ -104,9 +104,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBC36B16-DE46-4C6E-A6ED-9C66C3DB41B7}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="89.81640625" bestFit="1" customWidth="1"/>
@@ -424,24 +423,6 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C7" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C11" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -687,15 +668,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="398d2b5b-77f8-4c5f-a794-3d35ce849315">
@@ -704,6 +676,15 @@
     <TaxCatchAll xmlns="1c52e43a-7a2d-43c4-9ede-f251c929c0a1" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -726,14 +707,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{253E2BCE-BEE3-46CA-82C7-E211846F5250}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D118C015-E179-46FB-B6E8-2D926D65EB7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -742,4 +715,12 @@
     <ds:schemaRef ds:uri="1c52e43a-7a2d-43c4-9ede-f251c929c0a1"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{253E2BCE-BEE3-46CA-82C7-E211846F5250}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Re-export the Aciclovir example model with PK-Sim 13
The example project carries the Aciclovir simulation regenerated by PK-Sim 13 (from OSPSuite-R PR 2031). Its application path gained a `No formulation` segment, so the dose parameter now lives at `Events|IV 250mg 10min|No formulation|Application_1|ProtocolSchemaItem|Dose`. The example `Applications.xlsx`, `ProjectConfiguration.json`, the `utilities-config-json` snapshot, two scenario tests, and the sensitivity article use the new path. The function examples keep the old path because they load the Aciclovir model bundled with ospsuite, which is unchanged.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/TestProject/Configurations/Applications.xlsx
+++ b/inst/extdata/examples/TestProject/Configurations/Applications.xlsx
@@ -1,28 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RudolfEngelke\Documents\RStudio.wd\esqlabsR.worktrees\pi-workflow\inst\extdata\examples\TestProject\Configurations\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FB32BF-B241-40FB-8B38-44C19CC994C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7790" yWindow="760" windowWidth="27640" windowHeight="19270" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7790" yWindow="760" windowWidth="27640" windowHeight="19270" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Aciclovir_iv_250mg" sheetId="1" r:id="rId1"/>
-    <sheet name="Protocol_250mg" sheetId="2" r:id="rId2"/>
-    <sheet name="Protocol_500mg" sheetId="3" r:id="rId3"/>
+    <sheet name="Aciclovir_iv_250mg" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Protocol_250mg" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Protocol_500mg" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Container Path</t>
   </si>
@@ -43,22 +36,18 @@
   </si>
   <si>
     <t>Events|IV 250mg 10min|Application_1|ProtocolSchemaItem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Events|IV 250mg 10min|No formulation|Application_1|ProtocolSchemaItem</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -71,6 +60,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -90,22 +85,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Standard 2" xfId="1" xr:uid="{50F91E0E-941E-40F8-8246-13206B329C82}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -406,14 +397,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="56.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="56.54296875" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -427,14 +418,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="s">
@@ -443,18 +434,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="56.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="56.54296875" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -468,14 +460,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>6</v>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="s">
@@ -484,18 +476,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="51.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.7265625" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -509,14 +502,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>6</v>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>500</v>
       </c>
       <c r="D2" t="s">
@@ -525,5 +518,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>